<commit_message>
Remove BRK.B from financials sector
</commit_message>
<xml_diff>
--- a/data/csv/Financials.xlsx
+++ b/data/csv/Financials.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wfpin\Desktop\Projects\gravity\data\csv\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{896C5ED2-75B6-46B4-8AB3-261BBC4E062D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53C12CB7-E7B9-4C77-BCA3-1CFEC589C77A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{0A2BC399-7504-47C9-8AAF-BA3F26D4D14D}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="76">
   <si>
     <t>ACGL</t>
   </si>
@@ -81,9 +81,6 @@
   </si>
   <si>
     <t>BLK</t>
-  </si>
-  <si>
-    <t>BRK.B</t>
   </si>
   <si>
     <t>BRO</t>
@@ -638,12 +635,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{747BBAF4-5550-4E07-8496-B92A14B368F9}">
-  <dimension ref="A1:A77"/>
+  <dimension ref="A1:A76"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.35">
@@ -1019,11 +1016,6 @@
     <row r="76" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>74</v>
-      </c>
-    </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A77" t="s">
-        <v>75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Remove FISV (no description)
</commit_message>
<xml_diff>
--- a/data/csv/Financials.xlsx
+++ b/data/csv/Financials.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wfpin\Desktop\Projects\gravity\data\csv\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53C12CB7-E7B9-4C77-BCA3-1CFEC589C77A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D89955B-292E-41E7-8E70-1693D0EDF705}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{0A2BC399-7504-47C9-8AAF-BA3F26D4D14D}"/>
   </bookViews>

</xml_diff>